<commit_message>
test IK acc & add RCM GUI & add PS5 to control movement after RCM
</commit_message>
<xml_diff>
--- a/da_vinci_tool_integration/rounded_poses.xlsx
+++ b/da_vinci_tool_integration/rounded_poses.xlsx
@@ -1,15 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29122"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emckclac-my.sharepoint.com/personal/k24104475_kcl_ac_uk/Documents/Microsoft Teams Chat Files/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_B49E05B2AFF76FFC05FC9890E22D62B1F034520D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6EDE498-D642-4B88-B459-8F189013A2B7}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -43,7 +65,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -107,13 +129,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -151,7 +181,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -185,6 +215,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -219,9 +250,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -394,9 +426,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H51"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
@@ -429,13 +461,13 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>-0.068</v>
+        <v>-6.8000000000000005E-2</v>
       </c>
       <c r="C2">
-        <v>0.449</v>
+        <v>0.44900000000000001</v>
       </c>
       <c r="D2">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E2">
         <v>-0.5</v>
@@ -455,25 +487,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-0.075</v>
+        <v>-7.4999999999999997E-2</v>
       </c>
       <c r="C3">
-        <v>0.471</v>
+        <v>0.47099999999999997</v>
       </c>
       <c r="D3">
-        <v>1.021</v>
+        <v>1.0209999999999999</v>
       </c>
       <c r="E3">
-        <v>-0.612</v>
+        <v>-0.61199999999999999</v>
       </c>
       <c r="F3">
-        <v>0.612</v>
+        <v>0.61199999999999999</v>
       </c>
       <c r="G3">
-        <v>0.355</v>
+        <v>0.35499999999999998</v>
       </c>
       <c r="H3">
-        <v>0.355</v>
+        <v>0.35499999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -481,25 +513,25 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>-0.418</v>
+        <v>-0.41799999999999998</v>
       </c>
       <c r="C4">
-        <v>0.381</v>
+        <v>0.38100000000000001</v>
       </c>
       <c r="D4">
-        <v>0.881</v>
+        <v>0.88100000000000001</v>
       </c>
       <c r="E4">
-        <v>-0.678</v>
+        <v>-0.67800000000000005</v>
       </c>
       <c r="F4">
         <v>0.51</v>
       </c>
       <c r="G4">
-        <v>0.489</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="H4">
-        <v>0.201</v>
+        <v>0.20100000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -507,25 +539,25 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>-0.638</v>
+        <v>-0.63800000000000001</v>
       </c>
       <c r="C5">
-        <v>0.163</v>
+        <v>0.16300000000000001</v>
       </c>
       <c r="D5">
-        <v>0.721</v>
+        <v>0.72099999999999997</v>
       </c>
       <c r="E5">
-        <v>-0.702</v>
+        <v>-0.70199999999999996</v>
       </c>
       <c r="F5">
         <v>0.52</v>
       </c>
       <c r="G5">
-        <v>0.454</v>
+        <v>0.45400000000000001</v>
       </c>
       <c r="H5">
-        <v>0.174</v>
+        <v>0.17399999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -533,25 +565,25 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>-0.133</v>
+        <v>-0.13300000000000001</v>
       </c>
       <c r="C6">
-        <v>0.825</v>
+        <v>0.82499999999999996</v>
       </c>
       <c r="D6">
-        <v>0.711</v>
+        <v>0.71099999999999997</v>
       </c>
       <c r="E6">
-        <v>-0.585</v>
+        <v>-0.58499999999999996</v>
       </c>
       <c r="F6">
-        <v>0.652</v>
+        <v>0.65200000000000002</v>
       </c>
       <c r="G6">
-        <v>0.226</v>
+        <v>0.22600000000000001</v>
       </c>
       <c r="H6">
-        <v>0.425</v>
+        <v>0.42499999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -562,22 +594,22 @@
         <v>-0.437</v>
       </c>
       <c r="C7">
-        <v>0.775</v>
+        <v>0.77500000000000002</v>
       </c>
       <c r="D7">
-        <v>0.421</v>
+        <v>0.42099999999999999</v>
       </c>
       <c r="E7">
-        <v>-0.641</v>
+        <v>-0.64100000000000001</v>
       </c>
       <c r="F7">
-        <v>0.613</v>
+        <v>0.61299999999999999</v>
       </c>
       <c r="G7">
         <v>0.318</v>
       </c>
       <c r="H7">
-        <v>0.336</v>
+        <v>0.33600000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -585,25 +617,25 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>-0.487</v>
+        <v>-0.48699999999999999</v>
       </c>
       <c r="C8">
-        <v>0.738</v>
+        <v>0.73799999999999999</v>
       </c>
       <c r="D8">
-        <v>0.243</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="E8">
-        <v>-0.716</v>
+        <v>-0.71599999999999997</v>
       </c>
       <c r="F8">
         <v>0.314</v>
       </c>
       <c r="G8">
-        <v>0.615</v>
+        <v>0.61499999999999999</v>
       </c>
       <c r="H8">
-        <v>-0.099</v>
+        <v>-9.9000000000000005E-2</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -611,22 +643,22 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>-0.899</v>
+        <v>-0.89900000000000002</v>
       </c>
       <c r="C9">
-        <v>0.244</v>
+        <v>0.24399999999999999</v>
       </c>
       <c r="D9">
-        <v>0.5659999999999999</v>
+        <v>0.56599999999999995</v>
       </c>
       <c r="E9">
-        <v>-0.782</v>
+        <v>-0.78200000000000003</v>
       </c>
       <c r="F9">
-        <v>-0.001</v>
+        <v>-1E-3</v>
       </c>
       <c r="G9">
-        <v>0.603</v>
+        <v>0.60299999999999998</v>
       </c>
       <c r="H9">
         <v>0.156</v>
@@ -637,22 +669,22 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>-0.853</v>
+        <v>-0.85299999999999998</v>
       </c>
       <c r="C10">
-        <v>0.204</v>
+        <v>0.20399999999999999</v>
       </c>
       <c r="D10">
         <v>0.91</v>
       </c>
       <c r="E10">
-        <v>-0.856</v>
+        <v>-0.85599999999999998</v>
       </c>
       <c r="F10">
         <v>0.02</v>
       </c>
       <c r="G10">
-        <v>0.493</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="H10">
         <v>0.155</v>
@@ -663,25 +695,25 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>-0.735</v>
+        <v>-0.73499999999999999</v>
       </c>
       <c r="C11">
-        <v>-0.162</v>
+        <v>-0.16200000000000001</v>
       </c>
       <c r="D11">
-        <v>0.718</v>
+        <v>0.71799999999999997</v>
       </c>
       <c r="E11">
-        <v>-0.8169999999999999</v>
+        <v>-0.81699999999999995</v>
       </c>
       <c r="F11">
-        <v>0.257</v>
+        <v>0.25700000000000001</v>
       </c>
       <c r="G11">
-        <v>0.517</v>
+        <v>0.51700000000000002</v>
       </c>
       <c r="H11">
-        <v>0.012</v>
+        <v>1.2E-2</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -689,25 +721,25 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>-0.712</v>
+        <v>-0.71199999999999997</v>
       </c>
       <c r="C12">
-        <v>-0.322</v>
+        <v>-0.32200000000000001</v>
       </c>
       <c r="D12">
         <v>0.307</v>
       </c>
       <c r="E12">
-        <v>-0.8129999999999999</v>
+        <v>-0.81299999999999994</v>
       </c>
       <c r="F12">
-        <v>0.268</v>
+        <v>0.26800000000000002</v>
       </c>
       <c r="G12">
-        <v>0.517</v>
+        <v>0.51700000000000002</v>
       </c>
       <c r="H12">
-        <v>0.005</v>
+        <v>5.0000000000000001E-3</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -715,25 +747,25 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>-0.774</v>
+        <v>-0.77400000000000002</v>
       </c>
       <c r="C13">
-        <v>-0.331</v>
+        <v>-0.33100000000000002</v>
       </c>
       <c r="D13">
-        <v>0.802</v>
+        <v>0.80200000000000005</v>
       </c>
       <c r="E13">
-        <v>-0.782</v>
+        <v>-0.78200000000000003</v>
       </c>
       <c r="F13">
-        <v>0.028</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="G13">
-        <v>0.5629999999999999</v>
+        <v>0.56299999999999994</v>
       </c>
       <c r="H13">
-        <v>-0.267</v>
+        <v>-0.26700000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -741,25 +773,25 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>-0.582</v>
+        <v>-0.58199999999999996</v>
       </c>
       <c r="C14">
-        <v>-0.635</v>
+        <v>-0.63500000000000001</v>
       </c>
       <c r="D14">
-        <v>0.651</v>
+        <v>0.65100000000000002</v>
       </c>
       <c r="E14">
-        <v>-0.601</v>
+        <v>-0.60099999999999998</v>
       </c>
       <c r="F14">
         <v>-0.501</v>
       </c>
       <c r="G14">
-        <v>0.598</v>
+        <v>0.59799999999999998</v>
       </c>
       <c r="H14">
-        <v>0.177</v>
+        <v>0.17699999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -767,25 +799,25 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>-0.381</v>
+        <v>-0.38100000000000001</v>
       </c>
       <c r="C15">
-        <v>-0.797</v>
+        <v>-0.79700000000000004</v>
       </c>
       <c r="D15">
-        <v>0.464</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="E15">
         <v>-0.74</v>
       </c>
       <c r="F15">
-        <v>-0.346</v>
+        <v>-0.34599999999999997</v>
       </c>
       <c r="G15">
-        <v>0.575</v>
+        <v>0.57499999999999996</v>
       </c>
       <c r="H15">
-        <v>0.057</v>
+        <v>5.7000000000000002E-2</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -796,22 +828,22 @@
         <v>-0.309</v>
       </c>
       <c r="C16">
-        <v>-0.888</v>
+        <v>-0.88800000000000001</v>
       </c>
       <c r="D16">
-        <v>0.868</v>
+        <v>0.86799999999999999</v>
       </c>
       <c r="E16">
-        <v>-0.574</v>
+        <v>-0.57399999999999995</v>
       </c>
       <c r="F16">
-        <v>-0.642</v>
+        <v>-0.64200000000000002</v>
       </c>
       <c r="G16">
         <v>0.503</v>
       </c>
       <c r="H16">
-        <v>0.074</v>
+        <v>7.3999999999999996E-2</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -819,22 +851,22 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>-0.205</v>
+        <v>-0.20499999999999999</v>
       </c>
       <c r="C17">
         <v>-0.871</v>
       </c>
       <c r="D17">
-        <v>0.508</v>
+        <v>0.50800000000000001</v>
       </c>
       <c r="E17">
-        <v>-0.598</v>
+        <v>-0.59799999999999998</v>
       </c>
       <c r="F17">
-        <v>-0.554</v>
+        <v>-0.55400000000000005</v>
       </c>
       <c r="G17">
-        <v>0.234</v>
+        <v>0.23400000000000001</v>
       </c>
       <c r="H17">
         <v>-0.53</v>
@@ -845,25 +877,25 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>-0.007</v>
+        <v>-7.0000000000000001E-3</v>
       </c>
       <c r="C18">
-        <v>-0.945</v>
+        <v>-0.94499999999999995</v>
       </c>
       <c r="D18">
         <v>0.224</v>
       </c>
       <c r="E18">
-        <v>-0.636</v>
+        <v>-0.63600000000000001</v>
       </c>
       <c r="F18">
-        <v>-0.661</v>
+        <v>-0.66100000000000003</v>
       </c>
       <c r="G18">
         <v>0.09</v>
       </c>
       <c r="H18">
-        <v>-0.388</v>
+        <v>-0.38800000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -871,22 +903,22 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0.119</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="C19">
         <v>-1.02</v>
       </c>
       <c r="D19">
-        <v>0.391</v>
+        <v>0.39100000000000001</v>
       </c>
       <c r="E19">
-        <v>-0.404</v>
+        <v>-0.40400000000000003</v>
       </c>
       <c r="F19">
-        <v>-0.635</v>
+        <v>-0.63500000000000001</v>
       </c>
       <c r="G19">
-        <v>-0.206</v>
+        <v>-0.20599999999999999</v>
       </c>
       <c r="H19">
         <v>-0.626</v>
@@ -897,25 +929,25 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.531</v>
+        <v>0.53100000000000003</v>
       </c>
       <c r="C20">
-        <v>-0.794</v>
+        <v>-0.79400000000000004</v>
       </c>
       <c r="D20">
-        <v>0.506</v>
+        <v>0.50600000000000001</v>
       </c>
       <c r="E20">
-        <v>-0.617</v>
+        <v>-0.61699999999999999</v>
       </c>
       <c r="F20">
-        <v>-0.665</v>
+        <v>-0.66500000000000004</v>
       </c>
       <c r="G20">
-        <v>0.059</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="H20">
-        <v>-0.417</v>
+        <v>-0.41699999999999998</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -923,25 +955,805 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.848</v>
+        <v>0.84799999999999998</v>
       </c>
       <c r="C21">
-        <v>-0.138</v>
+        <v>-0.13800000000000001</v>
       </c>
       <c r="D21">
-        <v>0.801</v>
+        <v>0.80100000000000005</v>
       </c>
       <c r="E21">
         <v>-0.03</v>
       </c>
       <c r="F21">
-        <v>-0.8110000000000001</v>
+        <v>-0.81100000000000005</v>
       </c>
       <c r="G21">
         <v>-0.43</v>
       </c>
       <c r="H21">
-        <v>-0.396</v>
+        <v>-0.39600000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>0.52270746229999998</v>
+      </c>
+      <c r="C22">
+        <v>0.359760046</v>
+      </c>
+      <c r="D22">
+        <v>1.0956012011</v>
+      </c>
+      <c r="E22">
+        <v>-0.29013136029999997</v>
+      </c>
+      <c r="F22">
+        <v>0.64484405519999999</v>
+      </c>
+      <c r="G22">
+        <v>0.29013136029999997</v>
+      </c>
+      <c r="H22">
+        <v>0.64484405519999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>0.59433221820000004</v>
+      </c>
+      <c r="C23">
+        <v>0.3770657778</v>
+      </c>
+      <c r="D23">
+        <v>0.95284569259999996</v>
+      </c>
+      <c r="E23">
+        <v>-0.34584525230000002</v>
+      </c>
+      <c r="F23">
+        <v>0.76867324110000002</v>
+      </c>
+      <c r="G23">
+        <v>0.2207793891</v>
+      </c>
+      <c r="H23">
+        <v>0.49070280789999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>0.88013380770000005</v>
+      </c>
+      <c r="C24">
+        <v>0.1370627284</v>
+      </c>
+      <c r="D24">
+        <v>0.31091225150000001</v>
+      </c>
+      <c r="E24">
+        <v>-0.43685567380000001</v>
+      </c>
+      <c r="F24">
+        <v>0.70911514760000005</v>
+      </c>
+      <c r="G24">
+        <v>0.36980786919999997</v>
+      </c>
+      <c r="H24">
+        <v>0.41177102920000003</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>0.9396686554</v>
+      </c>
+      <c r="C25">
+        <v>0.105758369</v>
+      </c>
+      <c r="D25">
+        <v>0.52457624670000003</v>
+      </c>
+      <c r="E25">
+        <v>-0.16344228390000001</v>
+      </c>
+      <c r="F25">
+        <v>0.79838275910000001</v>
+      </c>
+      <c r="G25">
+        <v>-4.67674062E-2</v>
+      </c>
+      <c r="H25">
+        <v>0.57765454049999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>0.97338730100000004</v>
+      </c>
+      <c r="C26">
+        <v>0.1017098427</v>
+      </c>
+      <c r="D26">
+        <v>0.75453907249999996</v>
+      </c>
+      <c r="E26">
+        <v>-0.1699674129</v>
+      </c>
+      <c r="F26">
+        <v>0.59297615290000005</v>
+      </c>
+      <c r="G26">
+        <v>3.4145601000000001E-3</v>
+      </c>
+      <c r="H26">
+        <v>0.78706979749999995</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>1.0274889468999999</v>
+      </c>
+      <c r="C27">
+        <v>6.5938398199999998E-2</v>
+      </c>
+      <c r="D27">
+        <v>0.5841422677</v>
+      </c>
+      <c r="E27">
+        <v>-3.8042485700000003E-2</v>
+      </c>
+      <c r="F27">
+        <v>0.84392768139999996</v>
+      </c>
+      <c r="G27">
+        <v>-0.31018728020000003</v>
+      </c>
+      <c r="H27">
+        <v>0.43603089449999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>1.1023749113000001</v>
+      </c>
+      <c r="C28">
+        <v>-0.21433773640000001</v>
+      </c>
+      <c r="D28">
+        <v>0.50633823870000005</v>
+      </c>
+      <c r="E28">
+        <v>0.1197405607</v>
+      </c>
+      <c r="F28">
+        <v>0.67812263969999997</v>
+      </c>
+      <c r="G28">
+        <v>-0.5904066563</v>
+      </c>
+      <c r="H28">
+        <v>0.42098975179999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>0.97468340399999998</v>
+      </c>
+      <c r="C29">
+        <v>-0.51346492769999996</v>
+      </c>
+      <c r="D29">
+        <v>0.86875003579999999</v>
+      </c>
+      <c r="E29">
+        <v>0.1197405607</v>
+      </c>
+      <c r="F29">
+        <v>0.67812263969999997</v>
+      </c>
+      <c r="G29">
+        <v>-0.5904066563</v>
+      </c>
+      <c r="H29">
+        <v>0.42098975179999998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>0.81061142679999998</v>
+      </c>
+      <c r="C30">
+        <v>-0.65300583840000004</v>
+      </c>
+      <c r="D30">
+        <v>0.58225327729999998</v>
+      </c>
+      <c r="E30">
+        <v>-7.8582480499999996E-2</v>
+      </c>
+      <c r="F30">
+        <v>0.86920005079999996</v>
+      </c>
+      <c r="G30">
+        <v>-0.2300467789</v>
+      </c>
+      <c r="H30">
+        <v>0.430575192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>0.71403592819999995</v>
+      </c>
+      <c r="C31">
+        <v>-0.65863960980000003</v>
+      </c>
+      <c r="D31">
+        <v>0.31853404639999999</v>
+      </c>
+      <c r="E31">
+        <v>5.13589084E-2</v>
+      </c>
+      <c r="F31">
+        <v>0.76328426599999999</v>
+      </c>
+      <c r="G31">
+        <v>-0.47521296140000002</v>
+      </c>
+      <c r="H31">
+        <v>0.43466365340000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>0.84279233220000005</v>
+      </c>
+      <c r="C32">
+        <v>-0.61977839469999996</v>
+      </c>
+      <c r="D32">
+        <v>0.63431644440000001</v>
+      </c>
+      <c r="E32">
+        <v>0.60164380070000001</v>
+      </c>
+      <c r="F32">
+        <v>0.4725096822</v>
+      </c>
+      <c r="G32">
+        <v>5.1029734000000004E-3</v>
+      </c>
+      <c r="H32">
+        <v>0.64399832489999997</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>0.71490448709999999</v>
+      </c>
+      <c r="C33">
+        <v>-0.66542816159999996</v>
+      </c>
+      <c r="D33">
+        <v>0.32871770859999999</v>
+      </c>
+      <c r="E33">
+        <v>0.60164380070000001</v>
+      </c>
+      <c r="F33">
+        <v>0.4725096822</v>
+      </c>
+      <c r="G33">
+        <v>5.1029734000000004E-3</v>
+      </c>
+      <c r="H33">
+        <v>0.64399832489999997</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>0.71313554050000005</v>
+      </c>
+      <c r="C34">
+        <v>-0.60931611060000002</v>
+      </c>
+      <c r="D34">
+        <v>0.25966972109999997</v>
+      </c>
+      <c r="E34">
+        <v>1.9208092199999999E-2</v>
+      </c>
+      <c r="F34">
+        <v>0.76476901770000005</v>
+      </c>
+      <c r="G34">
+        <v>-0.49307516219999997</v>
+      </c>
+      <c r="H34">
+        <v>0.41429060699999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>0.48002123829999999</v>
+      </c>
+      <c r="C35">
+        <v>-0.85737043619999997</v>
+      </c>
+      <c r="D35">
+        <v>0.62800192830000001</v>
+      </c>
+      <c r="E35">
+        <v>0.44356840850000001</v>
+      </c>
+      <c r="F35">
+        <v>0.62328779700000003</v>
+      </c>
+      <c r="G35">
+        <v>-0.17711848020000001</v>
+      </c>
+      <c r="H35">
+        <v>0.61918401720000005</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>-0.17246827479999999</v>
+      </c>
+      <c r="C36">
+        <v>-0.68416905400000005</v>
+      </c>
+      <c r="D36">
+        <v>0.87834537030000004</v>
+      </c>
+      <c r="E36">
+        <v>0.8243818879</v>
+      </c>
+      <c r="F36">
+        <v>0.20168283579999999</v>
+      </c>
+      <c r="G36">
+        <v>-0.52054089309999996</v>
+      </c>
+      <c r="H36">
+        <v>9.3574881600000007E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>-0.40957295900000001</v>
+      </c>
+      <c r="C37">
+        <v>0.30071225759999998</v>
+      </c>
+      <c r="D37">
+        <v>0.66518050429999998</v>
+      </c>
+      <c r="E37">
+        <v>0.82396203280000002</v>
+      </c>
+      <c r="F37">
+        <v>7.7450349900000007E-2</v>
+      </c>
+      <c r="G37">
+        <v>-0.55284750459999998</v>
+      </c>
+      <c r="H37">
+        <v>-9.7202122200000005E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>-0.18654347960000001</v>
+      </c>
+      <c r="C38">
+        <v>0.50599414109999996</v>
+      </c>
+      <c r="D38">
+        <v>0.71472549439999999</v>
+      </c>
+      <c r="E38">
+        <v>0.83637946839999999</v>
+      </c>
+      <c r="F38">
+        <v>-6.8218924099999995E-2</v>
+      </c>
+      <c r="G38">
+        <v>-0.3364322186</v>
+      </c>
+      <c r="H38">
+        <v>-0.42735183240000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>0.30979639289999999</v>
+      </c>
+      <c r="C39">
+        <v>0.75198805329999996</v>
+      </c>
+      <c r="D39">
+        <v>0.49872004990000002</v>
+      </c>
+      <c r="E39">
+        <v>0.66816246509999999</v>
+      </c>
+      <c r="F39">
+        <v>-0.50768429039999996</v>
+      </c>
+      <c r="G39">
+        <v>-0.51356452699999999</v>
+      </c>
+      <c r="H39">
+        <v>-0.1790741384</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>0.31805142759999999</v>
+      </c>
+      <c r="C40">
+        <v>0.74661910529999997</v>
+      </c>
+      <c r="D40">
+        <v>0.81202793120000005</v>
+      </c>
+      <c r="E40">
+        <v>0.49623143669999997</v>
+      </c>
+      <c r="F40">
+        <v>-0.69357424970000003</v>
+      </c>
+      <c r="G40">
+        <v>-0.20111344749999999</v>
+      </c>
+      <c r="H40">
+        <v>-0.48193675279999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>0.64610791209999996</v>
+      </c>
+      <c r="C41">
+        <v>0.84858477119999998</v>
+      </c>
+      <c r="D41">
+        <v>0.43203669789999999</v>
+      </c>
+      <c r="E41">
+        <v>0.49623143669999997</v>
+      </c>
+      <c r="F41">
+        <v>-0.69357424970000003</v>
+      </c>
+      <c r="G41">
+        <v>-0.20111344749999999</v>
+      </c>
+      <c r="H41">
+        <v>-0.48193675279999998</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>0.70706069469999999</v>
+      </c>
+      <c r="C42">
+        <v>0.76333343980000001</v>
+      </c>
+      <c r="D42">
+        <v>0.38173660640000001</v>
+      </c>
+      <c r="E42">
+        <v>0.49623143669999997</v>
+      </c>
+      <c r="F42">
+        <v>-0.69357424970000003</v>
+      </c>
+      <c r="G42">
+        <v>-0.20111344749999999</v>
+      </c>
+      <c r="H42">
+        <v>-0.48193675279999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>0.72692358489999997</v>
+      </c>
+      <c r="C43">
+        <v>0.74324822430000004</v>
+      </c>
+      <c r="D43">
+        <v>0.75837934019999997</v>
+      </c>
+      <c r="E43">
+        <v>0.39764729139999999</v>
+      </c>
+      <c r="F43">
+        <v>-0.48715913300000002</v>
+      </c>
+      <c r="G43">
+        <v>-0.35856506230000001</v>
+      </c>
+      <c r="H43">
+        <v>-0.68991613389999995</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>0.99013733859999997</v>
+      </c>
+      <c r="C44">
+        <v>0.30540481209999998</v>
+      </c>
+      <c r="D44">
+        <v>0.76140612360000004</v>
+      </c>
+      <c r="E44">
+        <v>-0.13887722790000001</v>
+      </c>
+      <c r="F44">
+        <v>-0.60366547110000002</v>
+      </c>
+      <c r="G44">
+        <v>3.8481112599999999E-2</v>
+      </c>
+      <c r="H44">
+        <v>-0.78410506250000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>4.8656851100000002E-2</v>
+      </c>
+      <c r="C45">
+        <v>0.66734576229999998</v>
+      </c>
+      <c r="D45">
+        <v>1.1185747385</v>
+      </c>
+      <c r="E45">
+        <v>-0.55536878109999999</v>
+      </c>
+      <c r="F45">
+        <v>0.43768200280000003</v>
+      </c>
+      <c r="G45">
+        <v>0.43768203259999999</v>
+      </c>
+      <c r="H45">
+        <v>0.55536884070000003</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>8.7492614999999996E-2</v>
+      </c>
+      <c r="C46">
+        <v>0.82567638160000001</v>
+      </c>
+      <c r="D46">
+        <v>0.92500525710000003</v>
+      </c>
+      <c r="E46">
+        <v>-0.37512969969999999</v>
+      </c>
+      <c r="F46">
+        <v>0.54381054640000004</v>
+      </c>
+      <c r="G46">
+        <v>0.29563692209999998</v>
+      </c>
+      <c r="H46">
+        <v>0.69003385309999998</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>0.3871185184</v>
+      </c>
+      <c r="C47">
+        <v>0.42093449830000002</v>
+      </c>
+      <c r="D47">
+        <v>1.2022092341999999</v>
+      </c>
+      <c r="E47">
+        <v>-0.25978147979999999</v>
+      </c>
+      <c r="F47">
+        <v>0.65765762329999999</v>
+      </c>
+      <c r="G47">
+        <v>0.25978147979999999</v>
+      </c>
+      <c r="H47">
+        <v>0.65765762329999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>0.52959215640000001</v>
+      </c>
+      <c r="C48">
+        <v>0.50011175870000002</v>
+      </c>
+      <c r="D48">
+        <v>1.0248816012999999</v>
+      </c>
+      <c r="E48">
+        <v>-0.1210958213</v>
+      </c>
+      <c r="F48">
+        <v>0.69666045899999995</v>
+      </c>
+      <c r="G48">
+        <v>0.1210958362</v>
+      </c>
+      <c r="H48">
+        <v>0.69666045899999995</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>0.59316194060000005</v>
+      </c>
+      <c r="C49">
+        <v>0.14675366879999999</v>
+      </c>
+      <c r="D49">
+        <v>0.91806250810000001</v>
+      </c>
+      <c r="E49">
+        <v>0.1573064327</v>
+      </c>
+      <c r="F49">
+        <v>0.81482934949999997</v>
+      </c>
+      <c r="G49">
+        <v>-0.10576169940000001</v>
+      </c>
+      <c r="H49">
+        <v>0.54783403870000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>0.47218048569999999</v>
+      </c>
+      <c r="C50">
+        <v>7.2977662099999993E-2</v>
+      </c>
+      <c r="D50">
+        <v>1.1095689535</v>
+      </c>
+      <c r="E50">
+        <v>0.1573064327</v>
+      </c>
+      <c r="F50">
+        <v>0.81482934949999997</v>
+      </c>
+      <c r="G50">
+        <v>-0.10576169940000001</v>
+      </c>
+      <c r="H50">
+        <v>0.54783403870000003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>0.64545947309999996</v>
+      </c>
+      <c r="C51">
+        <v>0.11394536500000001</v>
+      </c>
+      <c r="D51">
+        <v>0.90089678760000003</v>
+      </c>
+      <c r="E51">
+        <v>0.1573064327</v>
+      </c>
+      <c r="F51">
+        <v>0.81482934949999997</v>
+      </c>
+      <c r="G51">
+        <v>-0.10576169940000001</v>
+      </c>
+      <c r="H51">
+        <v>0.54783403870000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>